<commit_message>
Align Stage 1.2 formulas with named-range notation
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013goKf7PnbigP71dxwEQt5X
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -1650,7 +1650,7 @@
         <v>52</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">'Cost Structure'!$B$39</f>
+        <f aca="false">SeasonProfit</f>
         <v>42775.1553877422</v>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
         <v>55</v>
       </c>
       <c r="B17" s="18" t="n">
-        <f aca="false">'Cost Structure'!$B$13</f>
+        <f aca="false">TotalLaborRequired</f>
         <v>5276.82284632822</v>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
         <v>56</v>
       </c>
       <c r="B18" s="18" t="n">
-        <f aca="false">'Cost Structure'!$B$17</f>
+        <f aca="false">TotalLaborCapacity</f>
         <v>6480</v>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
         <v>58</v>
       </c>
       <c r="B20" s="19" t="n">
-        <f aca="false">'Cost Structure'!$B$16</f>
+        <f aca="false">TempWorkersNeeded</f>
         <v>4</v>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
         <v>68</v>
       </c>
       <c r="B13" s="22" t="n">
-        <f aca="false">B10+B11+B12</f>
+        <f aca="false">TomatoLaborHours+CarrotLaborHours+MesclunLaborHours</f>
         <v>5276.82284632822</v>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
         <v>69</v>
       </c>
       <c r="B14" s="21" t="n">
-        <f aca="false">MIN(B13,FarmerHours)</f>
+        <f aca="false">MIN(TotalLaborRequired,FarmerHours)</f>
         <v>720</v>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
         <v>70</v>
       </c>
       <c r="B15" s="21" t="n">
-        <f aca="false">MAX(B13-FarmerHours,0)</f>
+        <f aca="false">MAX(TotalLaborRequired-FarmerHours,0)</f>
         <v>4556.82284632822</v>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
         <v>58</v>
       </c>
       <c r="B16" s="10" t="n">
-        <f aca="false">IF(B15=0,0,MIN(MaxTempWorkers,ROUNDUP(B15/TempWorkerHours,0)))</f>
+        <f aca="false">IF(TempLaborHoursNeeded=0,0,MIN(MaxTempWorkers,ROUNDUP(TempLaborHoursNeeded/TempWorkerHours,0)))</f>
         <v>4</v>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
         <v>71</v>
       </c>
       <c r="B17" s="21" t="n">
-        <f aca="false">FarmerHours+B16*TempWorkerHours</f>
+        <f aca="false">FarmerHours+TempWorkersNeeded*TempWorkerHours</f>
         <v>6480</v>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
         <v>72</v>
       </c>
       <c r="B18" s="21" t="n">
-        <f aca="false">B17-B13</f>
+        <f aca="false">TotalLaborCapacity-TotalLaborRequired</f>
         <v>1203.17715367179</v>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
         <v>74</v>
       </c>
       <c r="B21" s="23" t="n">
-        <f aca="false">B14*FarmerRate</f>
+        <f aca="false">FarmerHoursUsed*FarmerRate</f>
         <v>24998.4</v>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
         <v>75</v>
       </c>
       <c r="B22" s="23" t="n">
-        <f aca="false">B15*TempRate</f>
+        <f aca="false">TempLaborHoursNeeded*TempRate</f>
         <v>79106.4446122578</v>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
         <v>76</v>
       </c>
       <c r="B23" s="24" t="n">
-        <f aca="false">B21+B22</f>
+        <f aca="false">FarmerLaborCost+TempLaborCost</f>
         <v>104104.844612258</v>
       </c>
     </row>
@@ -1919,7 +1919,7 @@
         <v>77</v>
       </c>
       <c r="B24" s="25" t="n">
-        <f aca="false">IF(B13=0,0,B23/B13)</f>
+        <f aca="false">IF(TotalLaborRequired=0,0,TotalLaborCost/TotalLaborRequired)</f>
         <v>19.7286980525976</v>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
         <v>78</v>
       </c>
       <c r="B28" s="24" t="n">
-        <f aca="false">B25+B26+B27</f>
+        <f aca="false">TomatoFertilizerCost+CarrotFertilizerCost+MesclunFertilizerCost</f>
         <v>44000</v>
       </c>
     </row>
@@ -1973,7 +1973,7 @@
         <v>79</v>
       </c>
       <c r="B30" s="24" t="n">
-        <f aca="false">B29+B28+B23</f>
+        <f aca="false">FixedCosts+TotalFertilizerCost+TotalLaborCost</f>
         <v>168104.844612258</v>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
         <v>84</v>
       </c>
       <c r="B36" s="24" t="n">
-        <f aca="false">B33+B34+B35</f>
+        <f aca="false">TomatoRevenue+CarrotRevenue+MesclunRevenue</f>
         <v>210880</v>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
         <v>86</v>
       </c>
       <c r="B39" s="27" t="n">
-        <f aca="false">B36-B30</f>
+        <f aca="false">TotalRevenue-TotalCost</f>
         <v>42775.1553877422</v>
       </c>
     </row>

</xml_diff>